<commit_message>
fix: align v3 probes with production flow
</commit_message>
<xml_diff>
--- a/source_package/eval/specs/v3_1/02_正式评测50题_v3.1_真实路由.xlsx
+++ b/source_package/eval/specs/v3_1/02_正式评测50题_v3.1_真实路由.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="正式50题_v3" sheetId="1" r:id="R771102157a734d9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="答案与SQL_v3" sheetId="2" r:id="R9498ddb4ec344591"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前测与探针" sheetId="3" r:id="R37951a3938554b88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作答脚本" sheetId="4" r:id="R83f41324272d4761"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标口径" sheetId="5" r:id="R6b11c7a6d0204a34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="正式50题_v3" sheetId="1" r:id="R6b4a06eaadcf429a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="答案与SQL_v3" sheetId="2" r:id="Ra6886a590aa04803"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前测与探针" sheetId="3" r:id="R440afb065190405e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作答脚本" sheetId="4" r:id="Rf290b15392bc402f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标口径" sheetId="5" r:id="R50839800cf024795"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -754,12 +754,8 @@
       <x:c r="P5" s="30" t="str">
         <x:v>wrong</x:v>
       </x:c>
-      <x:c r="Q5" s="30" t="str">
-        <x:v>DP-01-A</x:v>
-      </x:c>
-      <x:c r="R5" s="30" t="str">
-        <x:v>correct</x:v>
-      </x:c>
+      <x:c r="Q5" s="30"/>
+      <x:c r="R5" s="30"/>
       <x:c r="S5" s="30" t="str">
         <x:v>diagnostic_probe</x:v>
       </x:c>
@@ -2475,12 +2471,8 @@
       <x:c r="P20" s="30" t="str">
         <x:v>wrong</x:v>
       </x:c>
-      <x:c r="Q20" s="30" t="str">
-        <x:v>DP-02-A</x:v>
-      </x:c>
-      <x:c r="R20" s="30" t="str">
-        <x:v>correct</x:v>
-      </x:c>
+      <x:c r="Q20" s="30"/>
+      <x:c r="R20" s="30"/>
       <x:c r="S20" s="30" t="str">
         <x:v>diagnostic_probe</x:v>
       </x:c>
@@ -4761,12 +4753,8 @@
       <x:c r="P40" s="30" t="str">
         <x:v>wrong</x:v>
       </x:c>
-      <x:c r="Q40" s="30" t="str">
-        <x:v>DP-03-A</x:v>
-      </x:c>
-      <x:c r="R40" s="30" t="str">
-        <x:v>correct</x:v>
-      </x:c>
+      <x:c r="Q40" s="30"/>
+      <x:c r="R40" s="30"/>
       <x:c r="S40" s="30" t="str">
         <x:v>diagnostic_probe</x:v>
       </x:c>
@@ -5352,12 +5340,8 @@
       <x:c r="P45" s="30" t="str">
         <x:v>wrong</x:v>
       </x:c>
-      <x:c r="Q45" s="30" t="str">
-        <x:v>DP-04-A</x:v>
-      </x:c>
-      <x:c r="R45" s="30" t="str">
-        <x:v>correct</x:v>
-      </x:c>
+      <x:c r="Q45" s="30"/>
+      <x:c r="R45" s="30"/>
       <x:c r="S45" s="30" t="str">
         <x:v>diagnostic_probe</x:v>
       </x:c>
@@ -5943,12 +5927,8 @@
       <x:c r="P50" s="30" t="str">
         <x:v>wrong</x:v>
       </x:c>
-      <x:c r="Q50" s="30" t="str">
-        <x:v>DP-05-A</x:v>
-      </x:c>
-      <x:c r="R50" s="30" t="str">
-        <x:v>correct</x:v>
-      </x:c>
+      <x:c r="Q50" s="30"/>
+      <x:c r="R50" s="30"/>
       <x:c r="S50" s="30" t="str">
         <x:v>diagnostic_probe</x:v>
       </x:c>
@@ -6502,7 +6482,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1c94a722e2347de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd44d2e72b3c84d52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9105,7 +9085,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R018ccd4fd0484a3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb45a39a833a4c3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9868,7 +9848,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02989d6e04a9451f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fe939b9f19e4e15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10021,7 +10001,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2ff44cf7ba743fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b03acb769fb4c86"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>